<commit_message>
feat(docs): integrate hero showcase screenshot SHOT-01 and expand screenshot inventory
</commit_message>
<xml_diff>
--- a/docs/SCREENSHOT-INVENTORY.xlsx
+++ b/docs/SCREENSHOT-INVENTORY.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -593,10 +593,14 @@
           <t>docs/images/warpai-hero-showcase.png</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr"/>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>docs/images/warpai-hero-showcase.png</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -613,7 +617,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>README.md / docs/USING-WARPAI-AGENTS.md</t>
+          <t>docs/worktree-mode.md / docs/using-warpai-agents.md</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -656,7 +660,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>README.md / docs/USING-WARPAI-AGENTS.md</t>
+          <t>docs/worktree-mode.md / docs/using.md</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1172,7 +1176,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>docs/USING-WARPAI-AGENTS.md (Part 3)</t>
+          <t>docs/project-mode.md / docs/using-warpai-agents.md</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1215,7 +1219,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>docs/USING-WARPAI-AGENTS.md (Part 4)</t>
+          <t>docs/worktree-mode.md / docs/using-warpai-agents.md</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1541,6 +1545,221 @@
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>SHOT-24</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>docs/install.md (Section 3)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Linux Desktop Native Interface</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Linux 桌面端原生界面：在 Linux（Ubuntu GNOME/Debian/Fedora）桌面运行 Warpai 原生应用，展示原生窗口阴影、垂直标签栏及 GPU 渲染终端命令行。</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>1440x810 (16:9)</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>docs/images/linux-desktop-native.png</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="n"/>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>SHOT-25</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>docs/cli-agents.md</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Multi-Agent CLI Ecosystem in Action</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>20+ 款 CLI 智能体生态：Warpai 窗口中多标签/分屏同时运行 Claude Code、OpenAI Codex、Antigravity、Gemini 等不同智能体 CLI，展示零配置状态感知与环境隔离。</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>1440x810 (16:9)</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>docs/images/cli-agents-ecosystem.png</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="n"/>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>SHOT-26</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>docs/mcp-api.md / docs/worktree-mode.md</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Continuous Dispatch &amp; Dynamic Supervision List</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>动态任务监督与随时派发：协同面板 Tasks 区域特写，展示主 Agent 动态监督列表接纳随时派发的多分支任务，呈现 in_progress 实时进展及完成后自动退出。</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>1200x650</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>docs/images/mcp-dynamic-task-supervision.png</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>SHOT-27</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>docs/project-mode.md (Step 3 &amp; Step 5)</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Structured Q&amp;A Protocol &amp; Shared Memory Context</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Project 模式智能体问答与共享记忆：展示跨 Agent 呼出的结构化问答卡片（warp_agent_ask 阻断性咨询）及下方共享全局事实契约（Shared Context）面板。</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>1100x650</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>docs/images/project-mode-qa-context.png</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>SHOT-28</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>docs/config.md</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Ink Pure Dark Theme Presentation</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Ink 纯黑经典暗色主题全景：展示 Warpai 切换至 Ink Pure Dark 主题下的深黑底色、高对比度霓虹/柔光语法高亮及暗调协同面板。</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>1440x810 (16:9)</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>docs/images/appearance-ink-pure-dark.png</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="n"/>
+      <c r="I29" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
feat(docs): integrate SHOT-19, overhaul agent systems benchmark matrix, and reorganize landing blocks
</commit_message>
<xml_diff>
--- a/docs/SCREENSHOT-INVENTORY.xlsx
+++ b/docs/SCREENSHOT-INVENTORY.xlsx
@@ -1371,10 +1371,14 @@
           <t>docs/images/data-usage-quota-footer.png</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr"/>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>docs/images/data-usage-quota-footer.png</t>
+        </is>
+      </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>